<commit_message>
Mise a jour du 08-09-2026 14:55:42.86
</commit_message>
<xml_diff>
--- a/contenu/Seconde.xlsx
+++ b/contenu/Seconde.xlsx
@@ -579,7 +579,14 @@
           <t>Encadrer un nombre</t>
         </is>
       </c>
-      <c r="F3" s="3" t="n"/>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>sJIXJT3fdcU</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>366</v>
+      </c>
       <c r="I3" s="3" t="n"/>
       <c r="L3" s="3" t="n"/>
       <c r="O3" s="3" t="n"/>
@@ -604,7 +611,14 @@
           <t>Arrondir un nombre</t>
         </is>
       </c>
-      <c r="F4" s="3" t="n"/>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>53VOST9yJfg</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>438</v>
+      </c>
     </row>
     <row r="5" ht="29.1" customHeight="1" s="1">
       <c r="A5" t="n">
@@ -884,8 +898,8 @@
     <col width="11.109375" customWidth="1" style="1" min="1" max="1"/>
     <col width="60" customWidth="1" style="1" min="2" max="2"/>
     <col width="2.6640625" customWidth="1" style="1" min="3" max="237"/>
-    <col width="11.109375" customWidth="1" style="1" min="238" max="239"/>
-    <col width="11.109375" customWidth="1" style="1" min="240" max="16384"/>
+    <col width="11.109375" customWidth="1" style="1" min="238" max="240"/>
+    <col width="11.109375" customWidth="1" style="1" min="241" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="59.1" customHeight="1" s="1">
@@ -1617,11 +1631,6 @@
         </is>
       </c>
       <c r="H2" s="2" t="n"/>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1635,11 +1644,6 @@
         </is>
       </c>
       <c r="H3" s="2" t="n"/>
-      <c r="Z3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1653,11 +1657,6 @@
         </is>
       </c>
       <c r="H4" s="2" t="n"/>
-      <c r="Z4" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1736,6 +1735,11 @@
         </is>
       </c>
       <c r="H10" s="2" t="n"/>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="H11" s="2" t="n"/>

</xml_diff>

<commit_message>
Mise a jour du 29-09-2026 15:45:18,17
</commit_message>
<xml_diff>
--- a/contenu/Seconde.xlsx
+++ b/contenu/Seconde.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Liste" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Plannification" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Calendrier" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="liste date semaine" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Liste" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plannification" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calendrier" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="liste date semaine" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -402,23 +402,23 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.21875" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.23046875" defaultRowHeight="14.6"/>
   <cols>
-    <col width="2.88671875" customWidth="1" style="1" min="1" max="1"/>
-    <col width="4.6640625" customWidth="1" style="1" min="2" max="2"/>
-    <col width="4.44140625" customWidth="1" style="1" min="3" max="3"/>
-    <col width="3.109375" customWidth="1" style="1" min="4" max="4"/>
-    <col width="44.109375" customWidth="1" style="1" min="5" max="5"/>
-    <col width="3.33203125" customWidth="1" style="1" min="7" max="7"/>
+    <col width="2.84375" customWidth="1" style="1" min="1" max="1"/>
+    <col width="4.69140625" customWidth="1" style="1" min="2" max="2"/>
+    <col width="4.4609375" customWidth="1" style="1" min="3" max="3"/>
+    <col width="3.07421875" customWidth="1" style="1" min="4" max="4"/>
+    <col width="44.07421875" customWidth="1" style="1" min="5" max="5"/>
+    <col width="3.3046875" customWidth="1" style="1" min="7" max="7"/>
     <col width="7" customWidth="1" style="1" min="8" max="8"/>
-    <col width="2.33203125" customWidth="1" style="1" min="10" max="10"/>
-    <col width="3.88671875" customWidth="1" style="1" min="11" max="11"/>
-    <col width="1.88671875" customWidth="1" style="1" min="13" max="13"/>
-    <col width="2.77734375" customWidth="1" style="1" min="14" max="14"/>
-    <col width="2.33203125" customWidth="1" style="1" min="16" max="17"/>
+    <col width="2.3046875" customWidth="1" style="1" min="10" max="10"/>
+    <col width="3.84375" customWidth="1" style="1" min="11" max="11"/>
+    <col width="1.84375" customWidth="1" style="1" min="13" max="13"/>
+    <col width="2.765625" customWidth="1" style="1" min="14" max="14"/>
+    <col width="2.3046875" customWidth="1" style="1" min="16" max="17"/>
     <col width="2" customWidth="1" style="1" min="19" max="19"/>
-    <col width="2.21875" customWidth="1" style="1" min="20" max="20"/>
-    <col width="18.21875" customWidth="1" style="1" min="21" max="21"/>
+    <col width="2.23046875" customWidth="1" style="1" min="20" max="20"/>
+    <col width="18.23046875" customWidth="1" style="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -528,7 +528,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="29.1" customHeight="1" s="1">
+    <row r="2" ht="29.15" customHeight="1" s="1">
       <c r="A2" t="n">
         <v>2</v>
       </c>
@@ -559,7 +559,7 @@
       <c r="I2" s="3" t="n"/>
       <c r="L2" s="3" t="n"/>
     </row>
-    <row r="3" ht="43.8" customHeight="1" s="1">
+    <row r="3" ht="43.85" customHeight="1" s="1">
       <c r="A3" t="n">
         <v>2</v>
       </c>
@@ -591,7 +591,7 @@
       <c r="L3" s="3" t="n"/>
       <c r="O3" s="3" t="n"/>
     </row>
-    <row r="4" ht="29.1" customHeight="1" s="1">
+    <row r="4" ht="29.15" customHeight="1" s="1">
       <c r="A4" t="n">
         <v>2</v>
       </c>
@@ -620,7 +620,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="5" ht="29.1" customHeight="1" s="1">
+    <row r="5" ht="29.15" customHeight="1" s="1">
       <c r="A5" t="n">
         <v>2</v>
       </c>
@@ -658,7 +658,7 @@
       </c>
       <c r="L5" s="3" t="n"/>
     </row>
-    <row r="6" ht="29.1" customHeight="1" s="1">
+    <row r="6" ht="29.15" customHeight="1" s="1">
       <c r="A6" t="n">
         <v>2</v>
       </c>
@@ -703,7 +703,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="7" ht="29.1" customHeight="1" s="1">
+    <row r="7" ht="29.15" customHeight="1" s="1">
       <c r="A7" t="n">
         <v>2</v>
       </c>
@@ -734,7 +734,7 @@
       <c r="I7" s="3" t="n"/>
       <c r="L7" s="3" t="n"/>
     </row>
-    <row r="8" ht="29.1" customHeight="1" s="1">
+    <row r="8" ht="29.15" customHeight="1" s="1">
       <c r="A8" t="n">
         <v>2</v>
       </c>
@@ -838,7 +838,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="11" ht="29.1" customHeight="1" s="1">
+    <row r="11" ht="29.15" customHeight="1" s="1">
       <c r="A11" t="n">
         <v>2</v>
       </c>
@@ -899,7 +899,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="12" ht="29.1" customHeight="1" s="1">
+    <row r="12" ht="29.15" customHeight="1" s="1">
       <c r="A12" t="n">
         <v>2</v>
       </c>
@@ -944,7 +944,7 @@
         <v>635</v>
       </c>
     </row>
-    <row r="13" ht="29.1" customHeight="1" s="1">
+    <row r="13" ht="29.15" customHeight="1" s="1">
       <c r="A13" t="n">
         <v>2</v>
       </c>
@@ -974,7 +974,7 @@
       </c>
       <c r="I13" s="3" t="n"/>
     </row>
-    <row r="14" ht="29.1" customHeight="1" s="1">
+    <row r="14" ht="29.15" customHeight="1" s="1">
       <c r="A14" t="n">
         <v>2</v>
       </c>
@@ -1019,7 +1019,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="15" ht="29.1" customHeight="1" s="1">
+    <row r="15" ht="29.15" customHeight="1" s="1">
       <c r="A15" t="n">
         <v>2</v>
       </c>
@@ -1073,17 +1073,199 @@
       </c>
       <c r="R15" s="3" t="n"/>
     </row>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19" ht="29.1" customHeight="1" s="1">
+    <row r="16">
+      <c r="A16" t="n">
+        <v>2</v>
+      </c>
+      <c r="B16" t="n">
+        <v>2</v>
+      </c>
+      <c r="C16" t="n">
+        <v>4</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2.SF2.4</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Développer puis réduire uen expression</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>SH1hQrsZGsk</t>
+        </is>
+      </c>
+      <c r="H16" t="n">
+        <v>263</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>YS-3JI_z2f0</t>
+        </is>
+      </c>
+      <c r="K16" t="n">
+        <v>520</v>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>o6qVMmA3oTQ</t>
+        </is>
+      </c>
+      <c r="N16" t="n">
+        <v>275</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>hly4i9QDUT0</t>
+        </is>
+      </c>
+      <c r="Q16" t="n">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>2</v>
+      </c>
+      <c r="B17" t="n">
+        <v>2</v>
+      </c>
+      <c r="C17" t="n">
+        <v>5</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2.SF2.5</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Utilliser les identités remarquables</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>z3RzvSo6m_g</t>
+        </is>
+      </c>
+      <c r="H17" t="n">
+        <v>469</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>U98Tk89SJ5M</t>
+        </is>
+      </c>
+      <c r="K17" t="n">
+        <v>517</v>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>bm2m0XOfcmU</t>
+        </is>
+      </c>
+      <c r="T17" t="n">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>2</v>
+      </c>
+      <c r="B18" t="n">
+        <v>2</v>
+      </c>
+      <c r="C18" t="n">
+        <v>6</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>2.SF2.6</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Factoriser une expression</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>1OOl4u2kIg8</t>
+        </is>
+      </c>
+      <c r="H18" t="n">
+        <v>769</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>UGTFELhE9Dw</t>
+        </is>
+      </c>
+      <c r="K18" t="n">
+        <v>351</v>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>08peWLwhIzc</t>
+        </is>
+      </c>
+      <c r="Q18" t="n">
+        <v>327</v>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>ujBZ1luBUJE</t>
+        </is>
+      </c>
+      <c r="T18" t="n">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="19" ht="29.15" customHeight="1" s="1">
+      <c r="A19" t="n">
+        <v>2</v>
+      </c>
+      <c r="B19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C19" t="n">
+        <v>7</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>2.SF2.7</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Résoudre une équation produit nul</t>
+        </is>
+      </c>
       <c r="F19" s="3" t="n"/>
       <c r="I19" s="3" t="n"/>
       <c r="L19" s="3" t="n"/>
       <c r="O19" s="3" t="n"/>
     </row>
-    <row r="20"/>
-    <row r="21" ht="43.8" customHeight="1" s="1">
+    <row r="20">
+      <c r="A20" t="n">
+        <v>2</v>
+      </c>
+      <c r="B20" t="n">
+        <v>2</v>
+      </c>
+      <c r="C20" t="n">
+        <v>8</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>2.SF2.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="43.85" customHeight="1" s="1">
       <c r="F21" s="3" t="n"/>
     </row>
   </sheetData>
@@ -1098,16 +1280,16 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:IC230"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.109375" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.07421875" defaultRowHeight="14.6"/>
   <cols>
-    <col width="11.109375" customWidth="1" style="1" min="1" max="1"/>
+    <col width="11.07421875" customWidth="1" style="1" min="1" max="1"/>
     <col width="60" customWidth="1" style="1" min="2" max="2"/>
-    <col width="2.6640625" customWidth="1" style="1" min="3" max="237"/>
-    <col width="11.109375" customWidth="1" style="1" min="238" max="243"/>
-    <col width="11.109375" customWidth="1" style="1" min="244" max="16384"/>
+    <col width="2.69140625" customWidth="1" style="1" min="3" max="237"/>
+    <col width="11.07421875" customWidth="1" style="1" min="238" max="244"/>
+    <col width="11.07421875" customWidth="1" style="1" min="245" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" ht="59.1" customHeight="1" s="1">
+    <row r="1" ht="59.15" customHeight="1" s="1">
       <c r="A1" t="inlineStr">
         <is>
           <t>Code</t>
@@ -2012,18 +2194,63 @@
       <c r="H15" s="2" t="n"/>
     </row>
     <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2.SF2.4</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Développer puis réduire uen expression</t>
+        </is>
+      </c>
       <c r="H16" s="2" t="n"/>
     </row>
     <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2.SF2.5</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Utilliser les identités remarquables</t>
+        </is>
+      </c>
       <c r="H17" s="2" t="n"/>
     </row>
     <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2.SF2.6</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Factoriser une expression</t>
+        </is>
+      </c>
       <c r="H18" s="2" t="n"/>
     </row>
     <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2.SF2.7</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Résoudre une équation produit nul</t>
+        </is>
+      </c>
       <c r="H19" s="2" t="n"/>
     </row>
     <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2.SF2.8</t>
+        </is>
+      </c>
       <c r="H20" s="2" t="n"/>
     </row>
     <row r="21">
@@ -2668,9 +2895,9 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AQ16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6"/>
   <cols>
-    <col width="3.6640625" customWidth="1" style="1" min="2" max="43"/>
+    <col width="3.69140625" customWidth="1" style="1" min="2" max="43"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2934,7 +3161,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B15"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">

</xml_diff>

<commit_message>
Mise a jour du 01-10-2026 14:21:35.58
</commit_message>
<xml_diff>
--- a/contenu/Seconde.xlsx
+++ b/contenu/Seconde.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\Autres ordinateurs\Mon ordinateur portable\Cours\Site\contenu\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maxence\Documents\Cours\Site\contenu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{827CBCB2-CB73-4254-9780-616B2E7A99EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CFC3439-E8E9-47DC-8B9F-4C6BD6B9DF23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Liste" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="120">
   <si>
     <t>Préfixe</t>
   </si>
@@ -385,6 +385,9 @@
   </si>
   <si>
     <t>RFjtdC3wiJY</t>
+  </si>
+  <si>
+    <t>xmtZS0GwV_Y</t>
   </si>
 </sst>
 </file>
@@ -711,26 +714,26 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:U21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.23046875" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.21875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="2.84375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="4.69140625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="4.4609375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="3.07421875" style="1" customWidth="1"/>
-    <col min="5" max="5" width="44.07421875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="3.3046875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="2.88671875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="4.6640625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="4.44140625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="3.109375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="44.109375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="3.33203125" style="1" customWidth="1"/>
     <col min="8" max="8" width="7" style="1" customWidth="1"/>
-    <col min="10" max="10" width="2.3046875" style="1" customWidth="1"/>
-    <col min="11" max="11" width="3.84375" style="1" customWidth="1"/>
-    <col min="13" max="13" width="1.84375" style="1" customWidth="1"/>
-    <col min="14" max="14" width="2.765625" style="1" customWidth="1"/>
-    <col min="16" max="17" width="2.3046875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="2.33203125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="3.88671875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="1.88671875" style="1" customWidth="1"/>
+    <col min="14" max="14" width="2.77734375" style="1" customWidth="1"/>
+    <col min="16" max="17" width="2.33203125" style="1" customWidth="1"/>
     <col min="19" max="19" width="2" style="1" customWidth="1"/>
-    <col min="20" max="20" width="2.23046875" style="1" customWidth="1"/>
-    <col min="21" max="21" width="18.23046875" style="1" customWidth="1"/>
+    <col min="20" max="20" width="2.21875" style="1" customWidth="1"/>
+    <col min="21" max="21" width="18.21875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -795,7 +798,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2</v>
       </c>
@@ -820,7 +823,7 @@
       <c r="I2" s="3"/>
       <c r="L2" s="3"/>
     </row>
-    <row r="3" spans="1:21" ht="43.85" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:21" ht="43.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -846,7 +849,7 @@
       <c r="L3" s="3"/>
       <c r="O3" s="3"/>
     </row>
-    <row r="4" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2</v>
       </c>
@@ -869,7 +872,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="5" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2</v>
       </c>
@@ -899,7 +902,7 @@
       </c>
       <c r="L5" s="3"/>
     </row>
-    <row r="6" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2</v>
       </c>
@@ -934,7 +937,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="7" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>2</v>
       </c>
@@ -959,7 +962,7 @@
       <c r="I7" s="3"/>
       <c r="L7" s="3"/>
     </row>
-    <row r="8" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>2</v>
       </c>
@@ -983,7 +986,7 @@
       </c>
       <c r="L8" s="3"/>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>2</v>
       </c>
@@ -1006,7 +1009,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>2</v>
       </c>
@@ -1041,7 +1044,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="11" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>2</v>
       </c>
@@ -1088,7 +1091,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="12" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>2</v>
       </c>
@@ -1123,7 +1126,7 @@
         <v>635</v>
       </c>
     </row>
-    <row r="13" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>2</v>
       </c>
@@ -1147,7 +1150,7 @@
       </c>
       <c r="I13" s="3"/>
     </row>
-    <row r="14" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>2</v>
       </c>
@@ -1182,7 +1185,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="15" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>2</v>
       </c>
@@ -1224,7 +1227,7 @@
       </c>
       <c r="R15" s="3"/>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>2</v>
       </c>
@@ -1265,7 +1268,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>2</v>
       </c>
@@ -1299,6 +1302,12 @@
       <c r="N17" s="1">
         <v>402</v>
       </c>
+      <c r="O17" t="s">
+        <v>119</v>
+      </c>
+      <c r="Q17" s="1">
+        <v>509</v>
+      </c>
       <c r="R17" t="s">
         <v>89</v>
       </c>
@@ -1306,7 +1315,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>2</v>
       </c>
@@ -1347,7 +1356,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="19" spans="1:20" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:20" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>2</v>
       </c>
@@ -1368,7 +1377,7 @@
       <c r="L19" s="3"/>
       <c r="O19" s="3"/>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>2</v>
       </c>
@@ -1382,7 +1391,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="21" spans="1:20" ht="43.85" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:20" ht="43.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="F21" s="3"/>
     </row>
   </sheetData>
@@ -1393,16 +1402,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:IC230"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.07421875" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.07421875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="11.109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="60" style="1" customWidth="1"/>
-    <col min="3" max="237" width="2.69140625" style="1" customWidth="1"/>
-    <col min="238" max="245" width="11.07421875" style="1" customWidth="1"/>
-    <col min="246" max="16384" width="11.07421875" style="1"/>
+    <col min="3" max="237" width="2.6640625" style="1" customWidth="1"/>
+    <col min="238" max="245" width="11.109375" style="1" customWidth="1"/>
+    <col min="246" max="16384" width="11.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:237" ht="59.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:237" ht="59.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -2115,7 +2124,7 @@
         <v>46570</v>
       </c>
     </row>
-    <row r="2" spans="1:237" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>21</v>
       </c>
@@ -2124,7 +2133,7 @@
       </c>
       <c r="H2" s="2"/>
     </row>
-    <row r="3" spans="1:237" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>24</v>
       </c>
@@ -2133,7 +2142,7 @@
       </c>
       <c r="H3" s="2"/>
     </row>
-    <row r="4" spans="1:237" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>27</v>
       </c>
@@ -2142,7 +2151,7 @@
       </c>
       <c r="H4" s="2"/>
     </row>
-    <row r="5" spans="1:237" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>30</v>
       </c>
@@ -2151,7 +2160,7 @@
       </c>
       <c r="H5" s="2"/>
     </row>
-    <row r="6" spans="1:237" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>34</v>
       </c>
@@ -2160,7 +2169,7 @@
       </c>
       <c r="H6" s="2"/>
     </row>
-    <row r="7" spans="1:237" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>39</v>
       </c>
@@ -2169,7 +2178,7 @@
       </c>
       <c r="H7" s="2"/>
     </row>
-    <row r="8" spans="1:237" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>42</v>
       </c>
@@ -2178,7 +2187,7 @@
       </c>
       <c r="H8" s="2"/>
     </row>
-    <row r="9" spans="1:237" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>45</v>
       </c>
@@ -2187,7 +2196,7 @@
       </c>
       <c r="H9" s="2"/>
     </row>
-    <row r="10" spans="1:237" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>48</v>
       </c>
@@ -2199,7 +2208,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="11" spans="1:237" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>53</v>
       </c>
@@ -2208,7 +2217,7 @@
       </c>
       <c r="H11" s="2"/>
     </row>
-    <row r="12" spans="1:237" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>60</v>
       </c>
@@ -2217,7 +2226,7 @@
       </c>
       <c r="H12" s="2"/>
     </row>
-    <row r="13" spans="1:237" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>65</v>
       </c>
@@ -2226,7 +2235,7 @@
       </c>
       <c r="H13" s="2"/>
     </row>
-    <row r="14" spans="1:237" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>68</v>
       </c>
@@ -2235,7 +2244,7 @@
       </c>
       <c r="H14" s="2"/>
     </row>
-    <row r="15" spans="1:237" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>73</v>
       </c>
@@ -2244,7 +2253,7 @@
       </c>
       <c r="H15" s="2"/>
     </row>
-    <row r="16" spans="1:237" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>79</v>
       </c>
@@ -2253,7 +2262,7 @@
       </c>
       <c r="H16" s="2"/>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>85</v>
       </c>
@@ -2262,7 +2271,7 @@
       </c>
       <c r="H17" s="2"/>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>90</v>
       </c>
@@ -2271,7 +2280,7 @@
       </c>
       <c r="H18" s="2"/>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>96</v>
       </c>
@@ -2280,640 +2289,640 @@
       </c>
       <c r="H19" s="2"/>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>98</v>
       </c>
       <c r="H20" s="2"/>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H21" s="2"/>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H22" s="2"/>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H23" s="2"/>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H24" s="2"/>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H25" s="2"/>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H26" s="2"/>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H27" s="2"/>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H28" s="2"/>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H29" s="2"/>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H30" s="2"/>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H31" s="2"/>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H32" s="2"/>
     </row>
-    <row r="33" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="33" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H33" s="2"/>
     </row>
-    <row r="34" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="34" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H34" s="2"/>
     </row>
-    <row r="35" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="35" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H35" s="2"/>
     </row>
-    <row r="36" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="36" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H36" s="2"/>
     </row>
-    <row r="37" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="37" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H37" s="2"/>
     </row>
-    <row r="38" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="38" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H38" s="2"/>
     </row>
-    <row r="39" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="39" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H39" s="2"/>
     </row>
-    <row r="40" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="40" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H40" s="2"/>
     </row>
-    <row r="41" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="41" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H41" s="2"/>
     </row>
-    <row r="42" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="42" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H42" s="2"/>
     </row>
-    <row r="43" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="43" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H43" s="2"/>
     </row>
-    <row r="44" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="44" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H44" s="2"/>
     </row>
-    <row r="45" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="45" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H45" s="2"/>
     </row>
-    <row r="46" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="46" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H46" s="2"/>
     </row>
-    <row r="47" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="47" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H47" s="2"/>
     </row>
-    <row r="48" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="48" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H48" s="2"/>
     </row>
-    <row r="49" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="49" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H49" s="2"/>
     </row>
-    <row r="50" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="50" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H50" s="2"/>
     </row>
-    <row r="51" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="51" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H51" s="2"/>
     </row>
-    <row r="52" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="52" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H52" s="2"/>
     </row>
-    <row r="53" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="53" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H53" s="2"/>
     </row>
-    <row r="54" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="54" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H54" s="2"/>
     </row>
-    <row r="55" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="55" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H55" s="2"/>
     </row>
-    <row r="56" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="56" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H56" s="2"/>
     </row>
-    <row r="57" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="57" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H57" s="2"/>
     </row>
-    <row r="58" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="58" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H58" s="2"/>
     </row>
-    <row r="59" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="59" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H59" s="2"/>
     </row>
-    <row r="60" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="60" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H60" s="2"/>
     </row>
-    <row r="61" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="61" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H61" s="2"/>
     </row>
-    <row r="62" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="62" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H62" s="2"/>
     </row>
-    <row r="63" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="63" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H63" s="2"/>
     </row>
-    <row r="64" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="64" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H64" s="2"/>
     </row>
-    <row r="65" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="65" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H65" s="2"/>
     </row>
-    <row r="66" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="66" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H66" s="2"/>
     </row>
-    <row r="67" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="67" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H67" s="2"/>
     </row>
-    <row r="68" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="68" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H68" s="2"/>
     </row>
-    <row r="69" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="69" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H69" s="2"/>
     </row>
-    <row r="70" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="70" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H70" s="2"/>
     </row>
-    <row r="71" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="71" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H71" s="2"/>
     </row>
-    <row r="72" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="72" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H72" s="2"/>
     </row>
-    <row r="73" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="73" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H73" s="2"/>
     </row>
-    <row r="74" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="74" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H74" s="2"/>
     </row>
-    <row r="75" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="75" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H75" s="2"/>
     </row>
-    <row r="76" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="76" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H76" s="2"/>
     </row>
-    <row r="77" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="77" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H77" s="2"/>
     </row>
-    <row r="78" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="78" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H78" s="2"/>
     </row>
-    <row r="79" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="79" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H79" s="2"/>
     </row>
-    <row r="80" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="80" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H80" s="2"/>
     </row>
-    <row r="81" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="81" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H81" s="2"/>
     </row>
-    <row r="82" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="82" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H82" s="2"/>
     </row>
-    <row r="83" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="83" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H83" s="2"/>
     </row>
-    <row r="84" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="84" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H84" s="2"/>
     </row>
-    <row r="85" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="85" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H85" s="2"/>
     </row>
-    <row r="86" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="86" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H86" s="2"/>
     </row>
-    <row r="87" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="87" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H87" s="2"/>
     </row>
-    <row r="88" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="88" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H88" s="2"/>
     </row>
-    <row r="89" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="89" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H89" s="2"/>
     </row>
-    <row r="90" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="90" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H90" s="2"/>
     </row>
-    <row r="91" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="91" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H91" s="2"/>
     </row>
-    <row r="92" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="92" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H92" s="2"/>
     </row>
-    <row r="93" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="93" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H93" s="2"/>
     </row>
-    <row r="94" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="94" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H94" s="2"/>
     </row>
-    <row r="95" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="95" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H95" s="2"/>
     </row>
-    <row r="96" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="96" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H96" s="2"/>
     </row>
-    <row r="97" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="97" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H97" s="2"/>
     </row>
-    <row r="98" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="98" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H98" s="2"/>
     </row>
-    <row r="99" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="99" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H99" s="2"/>
     </row>
-    <row r="100" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="100" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H100" s="2"/>
     </row>
-    <row r="101" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="101" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H101" s="2"/>
     </row>
-    <row r="102" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="102" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H102" s="2"/>
     </row>
-    <row r="103" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="103" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H103" s="2"/>
     </row>
-    <row r="104" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="104" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H104" s="2"/>
     </row>
-    <row r="105" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="105" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H105" s="2"/>
     </row>
-    <row r="106" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="106" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H106" s="2"/>
     </row>
-    <row r="107" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="107" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H107" s="2"/>
     </row>
-    <row r="108" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="108" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H108" s="2"/>
     </row>
-    <row r="109" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="109" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H109" s="2"/>
     </row>
-    <row r="110" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="110" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H110" s="2"/>
     </row>
-    <row r="111" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="111" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H111" s="2"/>
     </row>
-    <row r="112" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="112" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H112" s="2"/>
     </row>
-    <row r="113" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="113" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H113" s="2"/>
     </row>
-    <row r="114" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="114" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H114" s="2"/>
     </row>
-    <row r="115" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="115" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H115" s="2"/>
     </row>
-    <row r="116" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="116" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H116" s="2"/>
     </row>
-    <row r="117" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="117" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H117" s="2"/>
     </row>
-    <row r="118" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="118" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H118" s="2"/>
     </row>
-    <row r="119" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="119" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H119" s="2"/>
     </row>
-    <row r="120" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="120" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H120" s="2"/>
     </row>
-    <row r="121" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="121" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H121" s="2"/>
     </row>
-    <row r="122" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="122" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H122" s="2"/>
     </row>
-    <row r="123" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="123" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H123" s="2"/>
     </row>
-    <row r="124" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="124" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H124" s="2"/>
     </row>
-    <row r="125" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="125" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H125" s="2"/>
     </row>
-    <row r="126" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="126" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H126" s="2"/>
     </row>
-    <row r="127" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="127" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H127" s="2"/>
     </row>
-    <row r="128" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="128" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H128" s="2"/>
     </row>
-    <row r="129" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="129" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H129" s="2"/>
     </row>
-    <row r="130" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="130" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H130" s="2"/>
     </row>
-    <row r="131" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="131" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H131" s="2"/>
     </row>
-    <row r="132" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="132" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H132" s="2"/>
     </row>
-    <row r="133" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="133" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H133" s="2"/>
     </row>
-    <row r="134" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="134" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H134" s="2"/>
     </row>
-    <row r="135" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="135" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H135" s="2"/>
     </row>
-    <row r="136" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="136" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H136" s="2"/>
     </row>
-    <row r="137" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="137" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H137" s="2"/>
     </row>
-    <row r="138" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="138" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H138" s="2"/>
     </row>
-    <row r="139" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="139" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H139" s="2"/>
     </row>
-    <row r="140" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="140" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H140" s="2"/>
     </row>
-    <row r="141" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="141" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H141" s="2"/>
     </row>
-    <row r="142" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="142" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H142" s="2"/>
     </row>
-    <row r="143" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="143" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H143" s="2"/>
     </row>
-    <row r="144" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="144" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H144" s="2"/>
     </row>
-    <row r="145" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="145" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H145" s="2"/>
     </row>
-    <row r="146" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="146" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H146" s="2"/>
     </row>
-    <row r="147" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="147" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H147" s="2"/>
     </row>
-    <row r="148" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="148" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H148" s="2"/>
     </row>
-    <row r="149" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="149" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H149" s="2"/>
     </row>
-    <row r="150" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="150" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H150" s="2"/>
     </row>
-    <row r="151" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="151" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H151" s="2"/>
     </row>
-    <row r="152" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="152" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H152" s="2"/>
     </row>
-    <row r="153" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="153" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H153" s="2"/>
     </row>
-    <row r="154" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="154" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H154" s="2"/>
     </row>
-    <row r="155" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="155" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H155" s="2"/>
     </row>
-    <row r="156" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="156" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H156" s="2"/>
     </row>
-    <row r="157" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="157" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H157" s="2"/>
     </row>
-    <row r="158" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="158" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H158" s="2"/>
     </row>
-    <row r="159" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="159" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H159" s="2"/>
     </row>
-    <row r="160" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="160" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H160" s="2"/>
     </row>
-    <row r="161" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="161" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H161" s="2"/>
     </row>
-    <row r="162" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="162" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H162" s="2"/>
     </row>
-    <row r="163" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="163" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H163" s="2"/>
     </row>
-    <row r="164" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="164" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H164" s="2"/>
     </row>
-    <row r="165" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="165" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H165" s="2"/>
     </row>
-    <row r="166" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="166" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H166" s="2"/>
     </row>
-    <row r="167" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="167" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H167" s="2"/>
     </row>
-    <row r="168" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="168" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H168" s="2"/>
     </row>
-    <row r="169" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="169" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H169" s="2"/>
     </row>
-    <row r="170" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="170" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H170" s="2"/>
     </row>
-    <row r="171" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="171" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H171" s="2"/>
     </row>
-    <row r="172" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="172" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H172" s="2"/>
     </row>
-    <row r="173" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="173" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H173" s="2"/>
     </row>
-    <row r="174" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="174" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H174" s="2"/>
     </row>
-    <row r="175" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="175" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H175" s="2"/>
     </row>
-    <row r="176" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="176" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H176" s="2"/>
     </row>
-    <row r="177" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="177" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H177" s="2"/>
     </row>
-    <row r="178" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="178" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H178" s="2"/>
     </row>
-    <row r="179" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="179" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H179" s="2"/>
     </row>
-    <row r="180" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="180" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H180" s="2"/>
     </row>
-    <row r="181" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="181" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H181" s="2"/>
     </row>
-    <row r="182" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="182" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H182" s="2"/>
     </row>
-    <row r="183" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="183" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H183" s="2"/>
     </row>
-    <row r="184" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="184" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H184" s="2"/>
     </row>
-    <row r="185" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="185" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H185" s="2"/>
     </row>
-    <row r="186" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="186" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H186" s="2"/>
     </row>
-    <row r="187" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="187" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H187" s="2"/>
     </row>
-    <row r="188" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="188" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H188" s="2"/>
     </row>
-    <row r="189" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="189" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H189" s="2"/>
     </row>
-    <row r="190" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="190" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H190" s="2"/>
     </row>
-    <row r="191" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="191" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H191" s="2"/>
     </row>
-    <row r="192" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="192" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H192" s="2"/>
     </row>
-    <row r="193" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="193" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H193" s="2"/>
     </row>
-    <row r="194" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="194" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H194" s="2"/>
     </row>
-    <row r="195" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="195" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H195" s="2"/>
     </row>
-    <row r="196" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="196" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H196" s="2"/>
     </row>
-    <row r="197" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="197" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H197" s="2"/>
     </row>
-    <row r="198" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="198" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H198" s="2"/>
     </row>
-    <row r="199" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="199" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H199" s="2"/>
     </row>
-    <row r="200" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="200" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H200" s="2"/>
     </row>
-    <row r="201" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="201" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H201" s="2"/>
     </row>
-    <row r="202" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="202" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H202" s="2"/>
     </row>
-    <row r="203" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="203" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H203" s="2"/>
     </row>
-    <row r="204" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="204" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H204" s="2"/>
     </row>
-    <row r="205" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="205" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H205" s="2"/>
     </row>
-    <row r="206" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="206" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H206" s="2"/>
     </row>
-    <row r="207" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="207" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H207" s="2"/>
     </row>
-    <row r="208" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="208" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H208" s="2"/>
     </row>
-    <row r="209" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="209" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H209" s="2"/>
     </row>
-    <row r="210" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="210" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H210" s="2"/>
     </row>
-    <row r="211" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="211" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H211" s="2"/>
     </row>
-    <row r="212" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="212" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H212" s="2"/>
     </row>
-    <row r="213" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="213" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H213" s="2"/>
     </row>
-    <row r="214" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="214" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H214" s="2"/>
     </row>
-    <row r="215" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="215" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H215" s="2"/>
     </row>
-    <row r="216" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="216" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H216" s="2"/>
     </row>
-    <row r="217" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="217" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H217" s="2"/>
     </row>
-    <row r="218" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="218" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H218" s="2"/>
     </row>
-    <row r="219" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="219" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H219" s="2"/>
     </row>
-    <row r="220" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="220" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H220" s="2"/>
     </row>
-    <row r="221" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="221" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H221" s="2"/>
     </row>
-    <row r="222" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="222" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H222" s="2"/>
     </row>
-    <row r="223" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="223" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H223" s="2"/>
     </row>
-    <row r="224" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="224" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H224" s="2"/>
     </row>
-    <row r="225" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="225" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H225" s="2"/>
     </row>
-    <row r="226" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="226" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H226" s="2"/>
     </row>
-    <row r="227" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="227" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H227" s="2"/>
     </row>
-    <row r="228" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="228" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H228" s="2"/>
     </row>
-    <row r="229" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="229" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H229" s="2"/>
     </row>
-    <row r="230" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="230" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H230" s="2"/>
     </row>
   </sheetData>
@@ -2924,12 +2933,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:AQ16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="43" width="3.69140625" style="1" customWidth="1"/>
+    <col min="2" max="43" width="3.6640625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:43" x14ac:dyDescent="0.3">
       <c r="B1">
         <v>37</v>
       </c>
@@ -3057,77 +3066,77 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:43" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="3" spans="1:43" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="4" spans="1:43" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="5" spans="1:43" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="6" spans="1:43" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="7" spans="1:43" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="8" spans="1:43" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="1:43" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="10" spans="1:43" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="11" spans="1:43" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="12" spans="1:43" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="13" spans="1:43" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="14" spans="1:43" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="15" spans="1:43" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="16" spans="1:43" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>115</v>
       </c>
@@ -3140,9 +3149,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B15"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>116</v>
       </c>
@@ -3150,7 +3159,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>37</v>
       </c>
@@ -3158,7 +3167,7 @@
         <v>46272</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>37</v>
       </c>
@@ -3166,7 +3175,7 @@
         <v>46273</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>37</v>
       </c>
@@ -3174,7 +3183,7 @@
         <v>46274</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>37</v>
       </c>
@@ -3182,7 +3191,7 @@
         <v>46275</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>37</v>
       </c>
@@ -3190,7 +3199,7 @@
         <v>46276</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>37</v>
       </c>
@@ -3198,7 +3207,7 @@
         <v>46277</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>37</v>
       </c>
@@ -3206,7 +3215,7 @@
         <v>46278</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>38</v>
       </c>
@@ -3214,7 +3223,7 @@
         <v>46279</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>38</v>
       </c>
@@ -3222,7 +3231,7 @@
         <v>46280</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>38</v>
       </c>
@@ -3230,7 +3239,7 @@
         <v>46281</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>38</v>
       </c>
@@ -3238,7 +3247,7 @@
         <v>46282</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>38</v>
       </c>
@@ -3246,7 +3255,7 @@
         <v>46283</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>38</v>
       </c>
@@ -3254,7 +3263,7 @@
         <v>46284</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>38</v>
       </c>

</xml_diff>

<commit_message>
Mise a jour du 17-10-2026 12:45:22,91
</commit_message>
<xml_diff>
--- a/contenu/Seconde.xlsx
+++ b/contenu/Seconde.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maxence\Documents\Cours\Site\contenu\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\Autres ordinateurs\Mon ordinateur portable\Cours\Site\contenu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CFC3439-E8E9-47DC-8B9F-4C6BD6B9DF23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45E0E7F1-7511-42BB-BBBF-9AC7867B5516}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Liste" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="124">
   <si>
     <t>Préfixe</t>
   </si>
@@ -297,6 +297,12 @@
     <t>U98Tk89SJ5M</t>
   </si>
   <si>
+    <t>RFjtdC3wiJY</t>
+  </si>
+  <si>
+    <t>xmtZS0GwV_Y</t>
+  </si>
+  <si>
     <t>bm2m0XOfcmU</t>
   </si>
   <si>
@@ -324,6 +330,18 @@
     <t>Résoudre une équation produit nul</t>
   </si>
   <si>
+    <t>KoMyPeLRTWg</t>
+  </si>
+  <si>
+    <t>0_5Al9pcjZs</t>
+  </si>
+  <si>
+    <t>BNXJgiaRmdk</t>
+  </si>
+  <si>
+    <t>SeSJdEq-GWA</t>
+  </si>
+  <si>
     <t>2.SF2.8</t>
   </si>
   <si>
@@ -382,12 +400,6 @@
   </si>
   <si>
     <t>Date</t>
-  </si>
-  <si>
-    <t>RFjtdC3wiJY</t>
-  </si>
-  <si>
-    <t>xmtZS0GwV_Y</t>
   </si>
 </sst>
 </file>
@@ -714,26 +726,26 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:U21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.21875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.23046875" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="2.88671875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="4.6640625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="4.44140625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="3.109375" style="1" customWidth="1"/>
-    <col min="5" max="5" width="44.109375" style="1" customWidth="1"/>
-    <col min="7" max="7" width="3.33203125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="2.84375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="4.69140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="4.4609375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="3.07421875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="44.07421875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="3.3046875" style="1" customWidth="1"/>
     <col min="8" max="8" width="7" style="1" customWidth="1"/>
-    <col min="10" max="10" width="2.33203125" style="1" customWidth="1"/>
-    <col min="11" max="11" width="3.88671875" style="1" customWidth="1"/>
-    <col min="13" max="13" width="1.88671875" style="1" customWidth="1"/>
-    <col min="14" max="14" width="2.77734375" style="1" customWidth="1"/>
-    <col min="16" max="17" width="2.33203125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="2.3046875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="3.84375" style="1" customWidth="1"/>
+    <col min="13" max="13" width="1.84375" style="1" customWidth="1"/>
+    <col min="14" max="14" width="2.765625" style="1" customWidth="1"/>
+    <col min="16" max="17" width="2.3046875" style="1" customWidth="1"/>
     <col min="19" max="19" width="2" style="1" customWidth="1"/>
-    <col min="20" max="20" width="2.21875" style="1" customWidth="1"/>
-    <col min="21" max="21" width="18.21875" style="1" customWidth="1"/>
+    <col min="20" max="20" width="2.23046875" style="1" customWidth="1"/>
+    <col min="21" max="21" width="18.23046875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -798,7 +810,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2">
         <v>2</v>
       </c>
@@ -823,7 +835,7 @@
       <c r="I2" s="3"/>
       <c r="L2" s="3"/>
     </row>
-    <row r="3" spans="1:21" ht="43.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:21" ht="43.85" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A3">
         <v>2</v>
       </c>
@@ -849,7 +861,7 @@
       <c r="L3" s="3"/>
       <c r="O3" s="3"/>
     </row>
-    <row r="4" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A4">
         <v>2</v>
       </c>
@@ -872,7 +884,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="5" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5">
         <v>2</v>
       </c>
@@ -902,7 +914,7 @@
       </c>
       <c r="L5" s="3"/>
     </row>
-    <row r="6" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A6">
         <v>2</v>
       </c>
@@ -937,7 +949,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="7" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A7">
         <v>2</v>
       </c>
@@ -962,7 +974,7 @@
       <c r="I7" s="3"/>
       <c r="L7" s="3"/>
     </row>
-    <row r="8" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A8">
         <v>2</v>
       </c>
@@ -986,7 +998,7 @@
       </c>
       <c r="L8" s="3"/>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A9">
         <v>2</v>
       </c>
@@ -1009,7 +1021,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A10">
         <v>2</v>
       </c>
@@ -1044,7 +1056,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="11" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A11">
         <v>2</v>
       </c>
@@ -1091,7 +1103,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="12" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A12">
         <v>2</v>
       </c>
@@ -1126,7 +1138,7 @@
         <v>635</v>
       </c>
     </row>
-    <row r="13" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A13">
         <v>2</v>
       </c>
@@ -1150,7 +1162,7 @@
       </c>
       <c r="I13" s="3"/>
     </row>
-    <row r="14" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A14">
         <v>2</v>
       </c>
@@ -1185,7 +1197,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="15" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A15">
         <v>2</v>
       </c>
@@ -1227,7 +1239,7 @@
       </c>
       <c r="R15" s="3"/>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A16">
         <v>2</v>
       </c>
@@ -1268,7 +1280,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A17">
         <v>2</v>
       </c>
@@ -1297,25 +1309,25 @@
         <v>517</v>
       </c>
       <c r="L17" t="s">
-        <v>118</v>
-      </c>
-      <c r="N17" s="1">
+        <v>89</v>
+      </c>
+      <c r="N17">
         <v>402</v>
       </c>
       <c r="O17" t="s">
-        <v>119</v>
-      </c>
-      <c r="Q17" s="1">
+        <v>90</v>
+      </c>
+      <c r="Q17">
         <v>509</v>
       </c>
       <c r="R17" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="T17">
         <v>513</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A18">
         <v>2</v>
       </c>
@@ -1326,37 +1338,37 @@
         <v>6</v>
       </c>
       <c r="D18" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E18" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F18" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="H18">
         <v>769</v>
       </c>
       <c r="I18" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="K18">
         <v>351</v>
       </c>
       <c r="O18" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="Q18">
         <v>327</v>
       </c>
       <c r="R18" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="T18">
         <v>242</v>
       </c>
     </row>
-    <row r="19" spans="1:20" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:20" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A19">
         <v>2</v>
       </c>
@@ -1367,17 +1379,38 @@
         <v>7</v>
       </c>
       <c r="D19" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E19" t="s">
-        <v>97</v>
-      </c>
-      <c r="F19" s="3"/>
-      <c r="I19" s="3"/>
-      <c r="L19" s="3"/>
+        <v>99</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="H19">
+        <v>415</v>
+      </c>
+      <c r="I19" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="K19">
+        <v>482</v>
+      </c>
+      <c r="L19" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="N19">
+        <v>422</v>
+      </c>
       <c r="O19" s="3"/>
-    </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="R19" t="s">
+        <v>103</v>
+      </c>
+      <c r="T19" s="1">
+        <v>976</v>
+      </c>
+    </row>
+    <row r="20" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A20">
         <v>2</v>
       </c>
@@ -1388,10 +1421,10 @@
         <v>8</v>
       </c>
       <c r="D20" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="21" spans="1:20" ht="43.8" customHeight="1" x14ac:dyDescent="0.3">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="21" spans="1:20" ht="43.85" customHeight="1" x14ac:dyDescent="0.4">
       <c r="F21" s="3"/>
     </row>
   </sheetData>
@@ -1402,16 +1435,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:IC230"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.07421875" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="11.109375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="11.07421875" style="1" customWidth="1"/>
     <col min="2" max="2" width="60" style="1" customWidth="1"/>
-    <col min="3" max="237" width="2.6640625" style="1" customWidth="1"/>
-    <col min="238" max="245" width="11.109375" style="1" customWidth="1"/>
-    <col min="246" max="16384" width="11.109375" style="1"/>
+    <col min="3" max="237" width="2.69140625" style="1" customWidth="1"/>
+    <col min="238" max="246" width="11.07421875" style="1" customWidth="1"/>
+    <col min="247" max="16384" width="11.07421875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:237" ht="59.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:237" ht="59.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -2124,7 +2157,7 @@
         <v>46570</v>
       </c>
     </row>
-    <row r="2" spans="1:237" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:237" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>21</v>
       </c>
@@ -2133,7 +2166,7 @@
       </c>
       <c r="H2" s="2"/>
     </row>
-    <row r="3" spans="1:237" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:237" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>24</v>
       </c>
@@ -2142,7 +2175,7 @@
       </c>
       <c r="H3" s="2"/>
     </row>
-    <row r="4" spans="1:237" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:237" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>27</v>
       </c>
@@ -2151,7 +2184,7 @@
       </c>
       <c r="H4" s="2"/>
     </row>
-    <row r="5" spans="1:237" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:237" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>30</v>
       </c>
@@ -2160,7 +2193,7 @@
       </c>
       <c r="H5" s="2"/>
     </row>
-    <row r="6" spans="1:237" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:237" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>34</v>
       </c>
@@ -2169,7 +2202,7 @@
       </c>
       <c r="H6" s="2"/>
     </row>
-    <row r="7" spans="1:237" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:237" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>39</v>
       </c>
@@ -2178,7 +2211,7 @@
       </c>
       <c r="H7" s="2"/>
     </row>
-    <row r="8" spans="1:237" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:237" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>42</v>
       </c>
@@ -2187,7 +2220,7 @@
       </c>
       <c r="H8" s="2"/>
     </row>
-    <row r="9" spans="1:237" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:237" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>45</v>
       </c>
@@ -2196,7 +2229,7 @@
       </c>
       <c r="H9" s="2"/>
     </row>
-    <row r="10" spans="1:237" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:237" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>48</v>
       </c>
@@ -2205,10 +2238,10 @@
       </c>
       <c r="H10" s="2"/>
       <c r="Y10" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="11" spans="1:237" x14ac:dyDescent="0.3">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="11" spans="1:237" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>53</v>
       </c>
@@ -2217,7 +2250,7 @@
       </c>
       <c r="H11" s="2"/>
     </row>
-    <row r="12" spans="1:237" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:237" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>60</v>
       </c>
@@ -2226,7 +2259,7 @@
       </c>
       <c r="H12" s="2"/>
     </row>
-    <row r="13" spans="1:237" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:237" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>65</v>
       </c>
@@ -2235,7 +2268,7 @@
       </c>
       <c r="H13" s="2"/>
     </row>
-    <row r="14" spans="1:237" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:237" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>68</v>
       </c>
@@ -2244,7 +2277,7 @@
       </c>
       <c r="H14" s="2"/>
     </row>
-    <row r="15" spans="1:237" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:237" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>73</v>
       </c>
@@ -2253,7 +2286,7 @@
       </c>
       <c r="H15" s="2"/>
     </row>
-    <row r="16" spans="1:237" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:237" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>79</v>
       </c>
@@ -2262,7 +2295,7 @@
       </c>
       <c r="H16" s="2"/>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>85</v>
       </c>
@@ -2271,658 +2304,658 @@
       </c>
       <c r="H17" s="2"/>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B18" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="H18" s="2"/>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B19" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="H19" s="2"/>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="H20" s="2"/>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.4">
       <c r="H21" s="2"/>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.4">
       <c r="H22" s="2"/>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.4">
       <c r="H23" s="2"/>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.4">
       <c r="H24" s="2"/>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.4">
       <c r="H25" s="2"/>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.4">
       <c r="H26" s="2"/>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.4">
       <c r="H27" s="2"/>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.4">
       <c r="H28" s="2"/>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.4">
       <c r="H29" s="2"/>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.4">
       <c r="H30" s="2"/>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.4">
       <c r="H31" s="2"/>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.4">
       <c r="H32" s="2"/>
     </row>
-    <row r="33" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="33" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H33" s="2"/>
     </row>
-    <row r="34" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="34" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H34" s="2"/>
     </row>
-    <row r="35" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="35" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H35" s="2"/>
     </row>
-    <row r="36" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="36" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H36" s="2"/>
     </row>
-    <row r="37" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="37" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H37" s="2"/>
     </row>
-    <row r="38" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="38" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H38" s="2"/>
     </row>
-    <row r="39" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="39" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H39" s="2"/>
     </row>
-    <row r="40" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="40" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H40" s="2"/>
     </row>
-    <row r="41" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="41" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H41" s="2"/>
     </row>
-    <row r="42" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="42" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H42" s="2"/>
     </row>
-    <row r="43" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="43" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H43" s="2"/>
     </row>
-    <row r="44" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="44" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H44" s="2"/>
     </row>
-    <row r="45" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="45" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H45" s="2"/>
     </row>
-    <row r="46" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="46" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H46" s="2"/>
     </row>
-    <row r="47" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="47" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H47" s="2"/>
     </row>
-    <row r="48" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="48" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H48" s="2"/>
     </row>
-    <row r="49" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="49" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H49" s="2"/>
     </row>
-    <row r="50" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="50" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H50" s="2"/>
     </row>
-    <row r="51" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="51" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H51" s="2"/>
     </row>
-    <row r="52" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="52" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H52" s="2"/>
     </row>
-    <row r="53" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="53" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H53" s="2"/>
     </row>
-    <row r="54" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="54" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H54" s="2"/>
     </row>
-    <row r="55" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="55" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H55" s="2"/>
     </row>
-    <row r="56" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="56" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H56" s="2"/>
     </row>
-    <row r="57" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="57" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H57" s="2"/>
     </row>
-    <row r="58" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="58" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H58" s="2"/>
     </row>
-    <row r="59" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="59" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H59" s="2"/>
     </row>
-    <row r="60" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="60" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H60" s="2"/>
     </row>
-    <row r="61" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="61" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H61" s="2"/>
     </row>
-    <row r="62" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="62" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H62" s="2"/>
     </row>
-    <row r="63" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="63" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H63" s="2"/>
     </row>
-    <row r="64" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="64" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H64" s="2"/>
     </row>
-    <row r="65" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="65" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H65" s="2"/>
     </row>
-    <row r="66" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="66" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H66" s="2"/>
     </row>
-    <row r="67" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="67" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H67" s="2"/>
     </row>
-    <row r="68" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="68" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H68" s="2"/>
     </row>
-    <row r="69" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="69" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H69" s="2"/>
     </row>
-    <row r="70" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="70" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H70" s="2"/>
     </row>
-    <row r="71" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="71" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H71" s="2"/>
     </row>
-    <row r="72" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="72" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H72" s="2"/>
     </row>
-    <row r="73" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="73" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H73" s="2"/>
     </row>
-    <row r="74" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="74" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H74" s="2"/>
     </row>
-    <row r="75" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="75" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H75" s="2"/>
     </row>
-    <row r="76" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="76" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H76" s="2"/>
     </row>
-    <row r="77" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="77" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H77" s="2"/>
     </row>
-    <row r="78" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="78" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H78" s="2"/>
     </row>
-    <row r="79" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="79" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H79" s="2"/>
     </row>
-    <row r="80" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="80" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H80" s="2"/>
     </row>
-    <row r="81" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="81" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H81" s="2"/>
     </row>
-    <row r="82" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="82" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H82" s="2"/>
     </row>
-    <row r="83" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="83" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H83" s="2"/>
     </row>
-    <row r="84" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="84" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H84" s="2"/>
     </row>
-    <row r="85" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="85" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H85" s="2"/>
     </row>
-    <row r="86" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="86" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H86" s="2"/>
     </row>
-    <row r="87" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="87" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H87" s="2"/>
     </row>
-    <row r="88" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="88" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H88" s="2"/>
     </row>
-    <row r="89" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="89" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H89" s="2"/>
     </row>
-    <row r="90" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="90" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H90" s="2"/>
     </row>
-    <row r="91" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="91" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H91" s="2"/>
     </row>
-    <row r="92" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="92" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H92" s="2"/>
     </row>
-    <row r="93" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="93" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H93" s="2"/>
     </row>
-    <row r="94" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="94" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H94" s="2"/>
     </row>
-    <row r="95" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="95" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H95" s="2"/>
     </row>
-    <row r="96" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="96" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H96" s="2"/>
     </row>
-    <row r="97" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="97" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H97" s="2"/>
     </row>
-    <row r="98" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="98" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H98" s="2"/>
     </row>
-    <row r="99" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="99" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H99" s="2"/>
     </row>
-    <row r="100" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="100" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H100" s="2"/>
     </row>
-    <row r="101" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="101" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H101" s="2"/>
     </row>
-    <row r="102" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="102" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H102" s="2"/>
     </row>
-    <row r="103" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="103" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H103" s="2"/>
     </row>
-    <row r="104" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="104" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H104" s="2"/>
     </row>
-    <row r="105" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="105" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H105" s="2"/>
     </row>
-    <row r="106" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="106" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H106" s="2"/>
     </row>
-    <row r="107" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="107" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H107" s="2"/>
     </row>
-    <row r="108" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="108" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H108" s="2"/>
     </row>
-    <row r="109" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="109" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H109" s="2"/>
     </row>
-    <row r="110" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="110" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H110" s="2"/>
     </row>
-    <row r="111" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="111" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H111" s="2"/>
     </row>
-    <row r="112" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="112" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H112" s="2"/>
     </row>
-    <row r="113" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="113" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H113" s="2"/>
     </row>
-    <row r="114" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="114" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H114" s="2"/>
     </row>
-    <row r="115" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="115" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H115" s="2"/>
     </row>
-    <row r="116" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="116" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H116" s="2"/>
     </row>
-    <row r="117" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="117" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H117" s="2"/>
     </row>
-    <row r="118" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="118" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H118" s="2"/>
     </row>
-    <row r="119" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="119" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H119" s="2"/>
     </row>
-    <row r="120" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="120" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H120" s="2"/>
     </row>
-    <row r="121" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="121" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H121" s="2"/>
     </row>
-    <row r="122" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="122" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H122" s="2"/>
     </row>
-    <row r="123" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="123" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H123" s="2"/>
     </row>
-    <row r="124" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="124" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H124" s="2"/>
     </row>
-    <row r="125" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="125" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H125" s="2"/>
     </row>
-    <row r="126" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="126" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H126" s="2"/>
     </row>
-    <row r="127" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="127" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H127" s="2"/>
     </row>
-    <row r="128" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="128" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H128" s="2"/>
     </row>
-    <row r="129" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="129" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H129" s="2"/>
     </row>
-    <row r="130" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="130" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H130" s="2"/>
     </row>
-    <row r="131" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="131" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H131" s="2"/>
     </row>
-    <row r="132" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="132" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H132" s="2"/>
     </row>
-    <row r="133" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="133" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H133" s="2"/>
     </row>
-    <row r="134" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="134" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H134" s="2"/>
     </row>
-    <row r="135" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="135" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H135" s="2"/>
     </row>
-    <row r="136" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="136" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H136" s="2"/>
     </row>
-    <row r="137" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="137" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H137" s="2"/>
     </row>
-    <row r="138" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="138" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H138" s="2"/>
     </row>
-    <row r="139" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="139" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H139" s="2"/>
     </row>
-    <row r="140" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="140" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H140" s="2"/>
     </row>
-    <row r="141" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="141" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H141" s="2"/>
     </row>
-    <row r="142" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="142" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H142" s="2"/>
     </row>
-    <row r="143" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="143" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H143" s="2"/>
     </row>
-    <row r="144" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="144" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H144" s="2"/>
     </row>
-    <row r="145" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="145" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H145" s="2"/>
     </row>
-    <row r="146" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="146" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H146" s="2"/>
     </row>
-    <row r="147" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="147" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H147" s="2"/>
     </row>
-    <row r="148" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="148" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H148" s="2"/>
     </row>
-    <row r="149" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="149" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H149" s="2"/>
     </row>
-    <row r="150" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="150" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H150" s="2"/>
     </row>
-    <row r="151" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="151" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H151" s="2"/>
     </row>
-    <row r="152" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="152" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H152" s="2"/>
     </row>
-    <row r="153" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="153" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H153" s="2"/>
     </row>
-    <row r="154" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="154" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H154" s="2"/>
     </row>
-    <row r="155" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="155" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H155" s="2"/>
     </row>
-    <row r="156" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="156" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H156" s="2"/>
     </row>
-    <row r="157" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="157" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H157" s="2"/>
     </row>
-    <row r="158" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="158" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H158" s="2"/>
     </row>
-    <row r="159" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="159" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H159" s="2"/>
     </row>
-    <row r="160" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="160" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H160" s="2"/>
     </row>
-    <row r="161" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="161" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H161" s="2"/>
     </row>
-    <row r="162" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="162" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H162" s="2"/>
     </row>
-    <row r="163" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="163" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H163" s="2"/>
     </row>
-    <row r="164" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="164" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H164" s="2"/>
     </row>
-    <row r="165" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="165" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H165" s="2"/>
     </row>
-    <row r="166" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="166" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H166" s="2"/>
     </row>
-    <row r="167" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="167" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H167" s="2"/>
     </row>
-    <row r="168" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="168" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H168" s="2"/>
     </row>
-    <row r="169" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="169" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H169" s="2"/>
     </row>
-    <row r="170" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="170" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H170" s="2"/>
     </row>
-    <row r="171" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="171" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H171" s="2"/>
     </row>
-    <row r="172" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="172" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H172" s="2"/>
     </row>
-    <row r="173" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="173" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H173" s="2"/>
     </row>
-    <row r="174" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="174" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H174" s="2"/>
     </row>
-    <row r="175" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="175" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H175" s="2"/>
     </row>
-    <row r="176" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="176" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H176" s="2"/>
     </row>
-    <row r="177" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="177" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H177" s="2"/>
     </row>
-    <row r="178" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="178" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H178" s="2"/>
     </row>
-    <row r="179" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="179" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H179" s="2"/>
     </row>
-    <row r="180" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="180" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H180" s="2"/>
     </row>
-    <row r="181" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="181" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H181" s="2"/>
     </row>
-    <row r="182" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="182" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H182" s="2"/>
     </row>
-    <row r="183" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="183" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H183" s="2"/>
     </row>
-    <row r="184" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="184" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H184" s="2"/>
     </row>
-    <row r="185" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="185" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H185" s="2"/>
     </row>
-    <row r="186" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="186" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H186" s="2"/>
     </row>
-    <row r="187" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="187" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H187" s="2"/>
     </row>
-    <row r="188" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="188" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H188" s="2"/>
     </row>
-    <row r="189" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="189" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H189" s="2"/>
     </row>
-    <row r="190" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="190" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H190" s="2"/>
     </row>
-    <row r="191" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="191" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H191" s="2"/>
     </row>
-    <row r="192" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="192" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H192" s="2"/>
     </row>
-    <row r="193" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="193" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H193" s="2"/>
     </row>
-    <row r="194" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="194" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H194" s="2"/>
     </row>
-    <row r="195" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="195" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H195" s="2"/>
     </row>
-    <row r="196" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="196" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H196" s="2"/>
     </row>
-    <row r="197" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="197" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H197" s="2"/>
     </row>
-    <row r="198" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="198" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H198" s="2"/>
     </row>
-    <row r="199" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="199" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H199" s="2"/>
     </row>
-    <row r="200" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="200" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H200" s="2"/>
     </row>
-    <row r="201" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="201" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H201" s="2"/>
     </row>
-    <row r="202" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="202" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H202" s="2"/>
     </row>
-    <row r="203" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="203" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H203" s="2"/>
     </row>
-    <row r="204" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="204" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H204" s="2"/>
     </row>
-    <row r="205" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="205" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H205" s="2"/>
     </row>
-    <row r="206" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="206" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H206" s="2"/>
     </row>
-    <row r="207" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="207" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H207" s="2"/>
     </row>
-    <row r="208" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="208" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H208" s="2"/>
     </row>
-    <row r="209" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="209" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H209" s="2"/>
     </row>
-    <row r="210" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="210" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H210" s="2"/>
     </row>
-    <row r="211" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="211" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H211" s="2"/>
     </row>
-    <row r="212" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="212" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H212" s="2"/>
     </row>
-    <row r="213" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="213" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H213" s="2"/>
     </row>
-    <row r="214" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="214" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H214" s="2"/>
     </row>
-    <row r="215" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="215" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H215" s="2"/>
     </row>
-    <row r="216" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="216" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H216" s="2"/>
     </row>
-    <row r="217" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="217" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H217" s="2"/>
     </row>
-    <row r="218" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="218" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H218" s="2"/>
     </row>
-    <row r="219" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="219" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H219" s="2"/>
     </row>
-    <row r="220" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="220" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H220" s="2"/>
     </row>
-    <row r="221" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="221" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H221" s="2"/>
     </row>
-    <row r="222" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="222" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H222" s="2"/>
     </row>
-    <row r="223" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="223" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H223" s="2"/>
     </row>
-    <row r="224" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="224" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H224" s="2"/>
     </row>
-    <row r="225" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="225" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H225" s="2"/>
     </row>
-    <row r="226" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="226" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H226" s="2"/>
     </row>
-    <row r="227" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="227" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H227" s="2"/>
     </row>
-    <row r="228" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="228" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H228" s="2"/>
     </row>
-    <row r="229" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="229" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H229" s="2"/>
     </row>
-    <row r="230" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="230" spans="8:8" x14ac:dyDescent="0.4">
       <c r="H230" s="2"/>
     </row>
   </sheetData>
@@ -2933,12 +2966,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:AQ16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="43" width="3.6640625" style="1" customWidth="1"/>
+    <col min="2" max="43" width="3.69140625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:43" x14ac:dyDescent="0.4">
       <c r="B1">
         <v>37</v>
       </c>
@@ -2958,10 +2991,10 @@
         <v>42</v>
       </c>
       <c r="H1" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="I1" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="J1">
         <v>45</v>
@@ -2985,10 +3018,10 @@
         <v>51</v>
       </c>
       <c r="Q1" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="R1" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="S1">
         <v>1</v>
@@ -3009,10 +3042,10 @@
         <v>6</v>
       </c>
       <c r="Y1" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="Z1" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="AA1">
         <v>9</v>
@@ -3033,10 +3066,10 @@
         <v>14</v>
       </c>
       <c r="AG1" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="AH1" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="AI1">
         <v>17</v>
@@ -3066,79 +3099,79 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:43" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="3" spans="1:43" x14ac:dyDescent="0.3">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="3" spans="1:43" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="4" spans="1:43" x14ac:dyDescent="0.3">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="4" spans="1:43" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="5" spans="1:43" x14ac:dyDescent="0.3">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="5" spans="1:43" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="6" spans="1:43" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="6" spans="1:43" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="7" spans="1:43" x14ac:dyDescent="0.3">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="7" spans="1:43" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="8" spans="1:43" x14ac:dyDescent="0.3">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="8" spans="1:43" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="9" spans="1:43" x14ac:dyDescent="0.3">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="9" spans="1:43" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="10" spans="1:43" x14ac:dyDescent="0.3">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="10" spans="1:43" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="11" spans="1:43" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="11" spans="1:43" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="12" spans="1:43" x14ac:dyDescent="0.3">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="12" spans="1:43" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="13" spans="1:43" x14ac:dyDescent="0.3">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="13" spans="1:43" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="14" spans="1:43" x14ac:dyDescent="0.3">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="14" spans="1:43" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="15" spans="1:43" x14ac:dyDescent="0.3">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="15" spans="1:43" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="16" spans="1:43" x14ac:dyDescent="0.3">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="16" spans="1:43" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
     </row>
   </sheetData>
@@ -3149,17 +3182,17 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B15"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="B1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A2">
         <v>37</v>
       </c>
@@ -3167,7 +3200,7 @@
         <v>46272</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A3">
         <v>37</v>
       </c>
@@ -3175,7 +3208,7 @@
         <v>46273</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A4">
         <v>37</v>
       </c>
@@ -3183,7 +3216,7 @@
         <v>46274</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A5">
         <v>37</v>
       </c>
@@ -3191,7 +3224,7 @@
         <v>46275</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A6">
         <v>37</v>
       </c>
@@ -3199,7 +3232,7 @@
         <v>46276</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A7">
         <v>37</v>
       </c>
@@ -3207,7 +3240,7 @@
         <v>46277</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A8">
         <v>37</v>
       </c>
@@ -3215,7 +3248,7 @@
         <v>46278</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A9">
         <v>38</v>
       </c>
@@ -3223,7 +3256,7 @@
         <v>46279</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A10">
         <v>38</v>
       </c>
@@ -3231,7 +3264,7 @@
         <v>46280</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A11">
         <v>38</v>
       </c>
@@ -3239,7 +3272,7 @@
         <v>46281</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A12">
         <v>38</v>
       </c>
@@ -3247,7 +3280,7 @@
         <v>46282</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A13">
         <v>38</v>
       </c>
@@ -3255,7 +3288,7 @@
         <v>46283</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A14">
         <v>38</v>
       </c>
@@ -3263,7 +3296,7 @@
         <v>46284</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A15">
         <v>38</v>
       </c>

</xml_diff>